<commit_message>
docs: input template sheet images all carry sample data (dloads and dloads (2) get two surcharges) and stop a few rows past it; page states template version 27 and 4 load blocks per dloads sheet
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019MWct99sAN4cmZsDr6H3a8
</commit_message>
<xml_diff>
--- a/docs/usage/sample_sheets/sheets_joints.xlsx
+++ b/docs/usage/sample_sheets/sheets_joints.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/.claude/worktrees/joints-r1/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9855A05C-E080-7E4F-9B02-CD939BBA37C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{119A1861-00BF-3949-902B-66F34C8769AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4280" yWindow="2000" windowWidth="40460" windowHeight="22500" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4280" yWindow="2000" windowWidth="40460" windowHeight="22500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -629,7 +629,7 @@
     <t>* piezometric line 2 is only required for rapid drawdown analysis</t>
   </si>
   <si>
-    <t>Type optons</t>
+    <t>Type options</t>
   </si>
   <si>
     <t>True piezometric line: u = γw × vertical distance below the line (static head).</t>
@@ -638,7 +638,7 @@
     <t>phreatic</t>
   </si>
   <si>
-    <t xml:space="preserve"> Phreatic surface: static head reduced by cos² of the line's slope.</t>
+    <t>Phreatic surface: static head reduced by cos² of the line's slope.</t>
   </si>
   <si>
     <t>#</t>
@@ -3770,11 +3770,11 @@
       </c>
       <c r="H3" s="3" t="str">
         <f>IF($G3="","",IFERROR(VLOOKUP($G3,$AH$8:$AJ$11,2,0),""))</f>
-        <v/>
+        <v>Tangent</v>
       </c>
       <c r="I3" s="3" t="str">
         <f t="shared" ref="I3:I32" si="1">IF($G3="","",IFERROR(VLOOKUP($G3,$AH$8:$AJ$11,3,0),""))</f>
-        <v/>
+        <v>Active</v>
       </c>
       <c r="J3" s="3">
         <v>800.0</v>
@@ -3845,11 +3845,11 @@
       </c>
       <c r="H4" s="3" t="str">
         <f>IF($G4="","",IFERROR(VLOOKUP($G4,$AH$8:$AJ$11,2,0),""))</f>
-        <v/>
+        <v>Tangent</v>
       </c>
       <c r="I4" s="3" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Active</v>
       </c>
       <c r="J4" s="3">
         <v>800.0</v>
@@ -3914,11 +3914,11 @@
       </c>
       <c r="H5" s="3" t="str">
         <f>IF($G5="","",IFERROR(VLOOKUP($G5,$AH$8:$AJ$11,2,0),""))</f>
-        <v/>
+        <v>Tangent</v>
       </c>
       <c r="I5" s="3" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Active</v>
       </c>
       <c r="J5" s="3">
         <v>800.0</v>
@@ -3979,11 +3979,11 @@
       </c>
       <c r="H6" s="3" t="str">
         <f>IF($G6="","",IFERROR(VLOOKUP($G6,$AH$8:$AJ$11,2,0),""))</f>
-        <v/>
+        <v>Tangent</v>
       </c>
       <c r="I6" s="3" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Active</v>
       </c>
       <c r="J6" s="3">
         <v>800.0</v>
@@ -4041,11 +4041,11 @@
       </c>
       <c r="H7" s="3" t="str">
         <f>IF($G7="","",IFERROR(VLOOKUP($G7,$AH$8:$AJ$11,2,0),""))</f>
-        <v/>
+        <v>Tangent</v>
       </c>
       <c r="I7" s="3" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Active</v>
       </c>
       <c r="J7" s="3">
         <v>800.0</v>
@@ -4103,11 +4103,11 @@
       </c>
       <c r="H8" s="3" t="str">
         <f>IF($G8="","",IFERROR(VLOOKUP($G8,$AH$8:$AJ$11,2,0),""))</f>
-        <v/>
+        <v>Tangent</v>
       </c>
       <c r="I8" s="3" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Active</v>
       </c>
       <c r="J8" s="3">
         <v>800.0</v>
@@ -11687,6 +11687,20 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="Y6:Z6"/>
     <mergeCell ref="AQ4:AR4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
@@ -11703,20 +11717,6 @@
     <mergeCell ref="AH4:AI4"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="Y6:Z6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -13083,6 +13083,20 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="P7:Q7"/>
+    <mergeCell ref="AB7:AC7"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="S7:T7"/>
+    <mergeCell ref="M7:N7"/>
     <mergeCell ref="S4:T4"/>
     <mergeCell ref="AQ7:AR7"/>
     <mergeCell ref="AN4:AO4"/>
@@ -13099,20 +13113,6 @@
     <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="V4:W4"/>
     <mergeCell ref="V7:W7"/>
-    <mergeCell ref="AB7:AC7"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="S7:T7"/>
-    <mergeCell ref="M7:N7"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="P7:Q7"/>
   </mergeCells>
   <conditionalFormatting sqref="B6 A7:B7">
     <cfRule type="expression" dxfId="19" priority="1">
@@ -13190,8 +13190,8 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5 E5 H5 K5 N5 Q5 T5 W5 Z5 AC5 AF5 AI5 AL5 AO5 AR5" xr:uid="{00000000-0002-0000-0300-000000000000}">
-      <formula1>"material,ssr reduce,ssr hold,ssr elastic,refine"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5 E5 H5 K5 N5 Q5 T5 W5 Z5 AC5 AF5 AI5 AL5 AO5 AR5" xr:uid="{2C58C22E-BB25-6145-9297-FDBC71F3461D}">
+      <formula1>"material,ssr reduce,ssr hold,ssr elastic,refine,joints"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>